<commit_message>
Update Vendor Payment Template with new data
</commit_message>
<xml_diff>
--- a/data/Vendor_Payment_Template.xlsx
+++ b/data/Vendor_Payment_Template.xlsx
@@ -1,21 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Automation_eFMS_Vendor\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF9E9033-5A5B-42C3-AD02-89E3F4383AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30128"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C579ECF-95BA-48AC-83F1-AE309011AED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Vendor_Payment" sheetId="1" r:id="rId1"/>
+    <sheet name="VENDOR_PAYMENT" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -25,64 +36,64 @@
     <t>MST</t>
   </si>
   <si>
-    <t>Vendor Code</t>
-  </si>
-  <si>
-    <t>Vendor Name</t>
-  </si>
-  <si>
-    <t>Số Hợp Đồng</t>
-  </si>
-  <si>
-    <t>Hạn Hợp Đồng</t>
-  </si>
-  <si>
-    <t>Hạn Thanh toán</t>
-  </si>
-  <si>
-    <t>Dịch vụ</t>
+    <t>VENDOR CODE</t>
+  </si>
+  <si>
+    <t>VENDOR NAME</t>
+  </si>
+  <si>
+    <t>SỐ HỢP ĐỒNG</t>
+  </si>
+  <si>
+    <t>HẠN HỢP ĐỒNG</t>
+  </si>
+  <si>
+    <t>HẠN THANH TOÁN</t>
+  </si>
+  <si>
+    <t>DỊCH VỤ</t>
   </si>
   <si>
     <t>NCC</t>
   </si>
   <si>
-    <t>Số ĐNTT-FMS</t>
-  </si>
-  <si>
-    <t>Số Hóa Đơn/Bang kê</t>
-  </si>
-  <si>
-    <t>Ngày Hóa Đơn</t>
-  </si>
-  <si>
-    <t>Số tiền</t>
-  </si>
-  <si>
-    <t>Ngày Lập-FMS</t>
-  </si>
-  <si>
-    <t>Ngày duyệt-HOD</t>
-  </si>
-  <si>
-    <t>Ngày kế toán đã kiểm tra</t>
-  </si>
-  <si>
-    <t>Ghi chú (nếu bị thiếu chứng)</t>
-  </si>
-  <si>
-    <t>Ngày CK dự kiến</t>
-  </si>
-  <si>
-    <t>Over due date</t>
-  </si>
-  <si>
-    <t>Lý do chưa thanh toán</t>
-  </si>
-  <si>
-    <t>Số Báo Nợ</t>
-  </si>
-  <si>
-    <t>Tình Trạng</t>
+    <t>SỐ ĐNTT-FMS</t>
+  </si>
+  <si>
+    <t>SỐ HOÁ ĐƠN/BANG KÊ</t>
+  </si>
+  <si>
+    <t>NGÀY HOÁ ĐƠN</t>
+  </si>
+  <si>
+    <t>SỐ TIỀN</t>
+  </si>
+  <si>
+    <t>NGÀY LẬP - FMS</t>
+  </si>
+  <si>
+    <t>NGÀY DUYỆT - HOD</t>
+  </si>
+  <si>
+    <t>NGÀY KẾ TOÁN ĐÃ KIỂM TRA</t>
+  </si>
+  <si>
+    <t>GHI CHÚ (NẾU BỊ THIẾU CHỨNG)</t>
+  </si>
+  <si>
+    <t>NGÀY CK DỰ KIẾN</t>
+  </si>
+  <si>
+    <t>OVER DUE DATE</t>
+  </si>
+  <si>
+    <t>LÝ DO CHƯA THANH TOÁN</t>
+  </si>
+  <si>
+    <t>SỐ BÁO NỢ</t>
+  </si>
+  <si>
+    <t>TÌNH TRẠNG</t>
   </si>
   <si>
     <t>CHI HỘ</t>
@@ -92,31 +103,29 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="8"/>
+      <b/>
+      <sz val="12"/>
       <color rgb="FFFFFF00"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -129,13 +138,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC00000"/>
-        <bgColor rgb="FF000000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF275317"/>
-        <bgColor rgb="FF000000"/>
+        <fgColor theme="9" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -151,18 +160,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -193,39 +199,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -277,7 +283,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -388,6 +394,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -396,13 +409,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -467,31 +473,11 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -499,34 +485,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:V1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" customWidth="1"/>
-    <col min="3" max="3" width="43" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="36.44140625" style="4" customWidth="1"/>
-    <col min="10" max="10" width="13.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.44140625" style="4" customWidth="1"/>
-    <col min="14" max="14" width="11.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.77734375" style="4" customWidth="1"/>
-    <col min="16" max="16" width="24.33203125" style="4" customWidth="1"/>
-    <col min="17" max="17" width="10.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22.28515625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="24" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.5703125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="16.28515625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="24.5703125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="28.85546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="32.5703125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="18.85546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="19.140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="26.28515625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="15.5703125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="15.7109375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="16.85546875" style="1" customWidth="1"/>
+    <col min="23" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="15.75" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -593,7 +580,6 @@
       <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add api2-state.json for payment state management, enhance OneDrive integration with new upload functionality, and refactor payment synchronization logic
</commit_message>
<xml_diff>
--- a/data/Vendor_Payment_Template.xlsx
+++ b/data/Vendor_Payment_Template.xlsx
@@ -1,21 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Automation_eFMS_Vendor\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF9E9033-5A5B-42C3-AD02-89E3F4383AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30128"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C579ECF-95BA-48AC-83F1-AE309011AED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Vendor_Payment" sheetId="1" r:id="rId1"/>
+    <sheet name="VENDOR_PAYMENT" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -25,64 +36,64 @@
     <t>MST</t>
   </si>
   <si>
-    <t>Vendor Code</t>
-  </si>
-  <si>
-    <t>Vendor Name</t>
-  </si>
-  <si>
-    <t>Số Hợp Đồng</t>
-  </si>
-  <si>
-    <t>Hạn Hợp Đồng</t>
-  </si>
-  <si>
-    <t>Hạn Thanh toán</t>
-  </si>
-  <si>
-    <t>Dịch vụ</t>
+    <t>VENDOR CODE</t>
+  </si>
+  <si>
+    <t>VENDOR NAME</t>
+  </si>
+  <si>
+    <t>SỐ HỢP ĐỒNG</t>
+  </si>
+  <si>
+    <t>HẠN HỢP ĐỒNG</t>
+  </si>
+  <si>
+    <t>HẠN THANH TOÁN</t>
+  </si>
+  <si>
+    <t>DỊCH VỤ</t>
   </si>
   <si>
     <t>NCC</t>
   </si>
   <si>
-    <t>Số ĐNTT-FMS</t>
-  </si>
-  <si>
-    <t>Số Hóa Đơn/Bang kê</t>
-  </si>
-  <si>
-    <t>Ngày Hóa Đơn</t>
-  </si>
-  <si>
-    <t>Số tiền</t>
-  </si>
-  <si>
-    <t>Ngày Lập-FMS</t>
-  </si>
-  <si>
-    <t>Ngày duyệt-HOD</t>
-  </si>
-  <si>
-    <t>Ngày kế toán đã kiểm tra</t>
-  </si>
-  <si>
-    <t>Ghi chú (nếu bị thiếu chứng)</t>
-  </si>
-  <si>
-    <t>Ngày CK dự kiến</t>
-  </si>
-  <si>
-    <t>Over due date</t>
-  </si>
-  <si>
-    <t>Lý do chưa thanh toán</t>
-  </si>
-  <si>
-    <t>Số Báo Nợ</t>
-  </si>
-  <si>
-    <t>Tình Trạng</t>
+    <t>SỐ ĐNTT-FMS</t>
+  </si>
+  <si>
+    <t>SỐ HOÁ ĐƠN/BANG KÊ</t>
+  </si>
+  <si>
+    <t>NGÀY HOÁ ĐƠN</t>
+  </si>
+  <si>
+    <t>SỐ TIỀN</t>
+  </si>
+  <si>
+    <t>NGÀY LẬP - FMS</t>
+  </si>
+  <si>
+    <t>NGÀY DUYỆT - HOD</t>
+  </si>
+  <si>
+    <t>NGÀY KẾ TOÁN ĐÃ KIỂM TRA</t>
+  </si>
+  <si>
+    <t>GHI CHÚ (NẾU BỊ THIẾU CHỨNG)</t>
+  </si>
+  <si>
+    <t>NGÀY CK DỰ KIẾN</t>
+  </si>
+  <si>
+    <t>OVER DUE DATE</t>
+  </si>
+  <si>
+    <t>LÝ DO CHƯA THANH TOÁN</t>
+  </si>
+  <si>
+    <t>SỐ BÁO NỢ</t>
+  </si>
+  <si>
+    <t>TÌNH TRẠNG</t>
   </si>
   <si>
     <t>CHI HỘ</t>
@@ -92,31 +103,29 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="8"/>
+      <b/>
+      <sz val="12"/>
       <color rgb="FFFFFF00"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -129,13 +138,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC00000"/>
-        <bgColor rgb="FF000000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF275317"/>
-        <bgColor rgb="FF000000"/>
+        <fgColor theme="9" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -151,18 +160,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -193,39 +199,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -277,7 +283,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -388,6 +394,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -396,13 +409,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -467,31 +473,11 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -499,34 +485,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:V1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" customWidth="1"/>
-    <col min="3" max="3" width="43" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="36.44140625" style="4" customWidth="1"/>
-    <col min="10" max="10" width="13.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.44140625" style="4" customWidth="1"/>
-    <col min="14" max="14" width="11.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.77734375" style="4" customWidth="1"/>
-    <col min="16" max="16" width="24.33203125" style="4" customWidth="1"/>
-    <col min="17" max="17" width="10.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22.28515625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="24" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.5703125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="16.28515625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="24.5703125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="28.85546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="32.5703125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="18.85546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="19.140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="26.28515625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="15.5703125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="15.7109375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="16.85546875" style="1" customWidth="1"/>
+    <col min="23" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="15.75" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -593,7 +580,6 @@
       <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Enhance API response handling by adding support for API 3, including new response structure and approval information retrieval. Update last run timestamp in api2-state.json and improve payment synchronization logic with settlement approval data.
</commit_message>
<xml_diff>
--- a/data/Vendor_Payment_Template.xlsx
+++ b/data/Vendor_Payment_Template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C579ECF-95BA-48AC-83F1-AE309011AED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366BF723-4551-4D2E-88B4-FFB3E04DF25C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENDOR_PAYMENT" sheetId="1" r:id="rId1"/>
@@ -103,7 +103,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -113,7 +113,7 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,14 +121,14 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="11"/>
       <color rgb="FFFFFF00"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -147,8 +147,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -156,20 +162,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -189,9 +216,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -229,7 +256,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -335,7 +362,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -477,7 +504,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -486,102 +513,103 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.5703125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="22.28515625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="24" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.5703125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16.28515625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="24.5703125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="28.85546875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="32.5703125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="18.85546875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="19.140625" style="1" customWidth="1"/>
-    <col min="19" max="19" width="26.28515625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="15.5703125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="15.7109375" style="1" customWidth="1"/>
-    <col min="22" max="22" width="16.85546875" style="1" customWidth="1"/>
-    <col min="23" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.88671875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="20.5546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="21.88671875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="49.109375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="18.88671875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="20.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="16.33203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="18.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="20" style="1" customWidth="1"/>
+    <col min="15" max="15" width="25.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="32.5546875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="18.88671875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="19.109375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="26.33203125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="15.5546875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="15.6640625" style="1" customWidth="1"/>
+    <col min="22" max="22" width="16.88671875" style="1" customWidth="1"/>
+    <col min="23" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:22" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="3" t="s">
         <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement API 4 response handling by adding new data structure and synchronization logic. Update last run timestamps in api2-state.json and api3-response.json, and enhance payment synchronization with invoice date retrieval. Remove temporary files and improve overall data management.
</commit_message>
<xml_diff>
--- a/data/Vendor_Payment_Template.xlsx
+++ b/data/Vendor_Payment_Template.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366BF723-4551-4D2E-88B4-FFB3E04DF25C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95348B2A-ABBE-4E45-99EE-51FD0B81B1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENDOR_PAYMENT" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Sort data insert file
</commit_message>
<xml_diff>
--- a/data/Vendor_Payment_Template.xlsx
+++ b/data/Vendor_Payment_Template.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95348B2A-ABBE-4E45-99EE-51FD0B81B1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C8E710D-49BC-4163-821D-7D8A8CE3156C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENDOR_PAYMENT" sheetId="1" r:id="rId1"/>
@@ -515,8 +515,8 @@
   <dimension ref="A1:V1"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23.88671875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.21875" style="2" customWidth="1"/>
     <col min="3" max="3" width="15.6640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="20.33203125" style="2" customWidth="1"/>
     <col min="5" max="5" width="20.5546875" style="2" customWidth="1"/>

</xml_diff>

<commit_message>
Update API response and state files with new last run timestamps, settlement counts, and enhanced payment data structure. Add new API response files for improved data handling and synchronization.
</commit_message>
<xml_diff>
--- a/data/Vendor_Payment_Template.xlsx
+++ b/data/Vendor_Payment_Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C8E710D-49BC-4163-821D-7D8A8CE3156C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BA5777-A033-4D6F-B604-4A9A1E497330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>MST</t>
   </si>
@@ -57,46 +57,49 @@
     <t>NCC</t>
   </si>
   <si>
+    <t>SỐ HOÁ ĐƠN/BANG KÊ</t>
+  </si>
+  <si>
+    <t>NGÀY HOÁ ĐƠN</t>
+  </si>
+  <si>
+    <t>NGÀY LẬP - FMS</t>
+  </si>
+  <si>
+    <t>NGÀY DUYỆT - HOD</t>
+  </si>
+  <si>
+    <t>NGÀY KẾ TOÁN ĐÃ KIỂM TRA</t>
+  </si>
+  <si>
+    <t>GHI CHÚ (NẾU BỊ THIẾU CHỨNG)</t>
+  </si>
+  <si>
+    <t>NGÀY CK DỰ KIẾN</t>
+  </si>
+  <si>
+    <t>OVER DUE DATE</t>
+  </si>
+  <si>
+    <t>LÝ DO CHƯA THANH TOÁN</t>
+  </si>
+  <si>
+    <t>SỐ BÁO NỢ</t>
+  </si>
+  <si>
+    <t>TÌNH TRẠNG</t>
+  </si>
+  <si>
+    <t>CHI HỘ</t>
+  </si>
+  <si>
+    <t>GROUP EFMS</t>
+  </si>
+  <si>
     <t>SỐ ĐNTT-FMS</t>
   </si>
   <si>
-    <t>SỐ HOÁ ĐƠN/BANG KÊ</t>
-  </si>
-  <si>
-    <t>NGÀY HOÁ ĐƠN</t>
-  </si>
-  <si>
-    <t>SỐ TIỀN</t>
-  </si>
-  <si>
-    <t>NGÀY LẬP - FMS</t>
-  </si>
-  <si>
-    <t>NGÀY DUYỆT - HOD</t>
-  </si>
-  <si>
-    <t>NGÀY KẾ TOÁN ĐÃ KIỂM TRA</t>
-  </si>
-  <si>
-    <t>GHI CHÚ (NẾU BỊ THIẾU CHỨNG)</t>
-  </si>
-  <si>
-    <t>NGÀY CK DỰ KIẾN</t>
-  </si>
-  <si>
-    <t>OVER DUE DATE</t>
-  </si>
-  <si>
-    <t>LÝ DO CHƯA THANH TOÁN</t>
-  </si>
-  <si>
-    <t>SỐ BÁO NỢ</t>
-  </si>
-  <si>
-    <t>TÌNH TRẠNG</t>
-  </si>
-  <si>
-    <t>CHI HỘ</t>
+    <t>SỐ TIỀN99</t>
   </si>
 </sst>
 </file>
@@ -512,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" style="1" customWidth="1"/>
@@ -522,25 +525,26 @@
     <col min="5" max="5" width="20.5546875" style="2" customWidth="1"/>
     <col min="6" max="6" width="21.88671875" style="2" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="49.109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="18.88671875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="4.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.77734375" style="1" customWidth="1"/>
     <col min="10" max="10" width="20.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22.109375" style="1" customWidth="1"/>
     <col min="12" max="12" width="16.33203125" style="1" customWidth="1"/>
     <col min="13" max="13" width="18.6640625" style="1" customWidth="1"/>
     <col min="14" max="14" width="20" style="1" customWidth="1"/>
     <col min="15" max="15" width="25.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="32.5546875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="18.88671875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="19.109375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="26.33203125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="15.5546875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="15.6640625" style="1" customWidth="1"/>
-    <col min="22" max="22" width="16.88671875" style="1" customWidth="1"/>
-    <col min="23" max="16384" width="9.109375" style="1"/>
+    <col min="16" max="16" width="14.44140625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="32.5546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="18.88671875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="19.109375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="26.33203125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="15.5546875" style="1" customWidth="1"/>
+    <col min="22" max="22" width="15.6640625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="16.88671875" style="1" customWidth="1"/>
+    <col min="24" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -566,46 +570,49 @@
         <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="P1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="R1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="T1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update API response and state files with new last run timestamps and settlement counts. Add new payment entries with enhanced data structure for improved synchronization and management. Remove outdated entries to streamline data handling.
</commit_message>
<xml_diff>
--- a/data/Vendor_Payment_Template.xlsx
+++ b/data/Vendor_Payment_Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BA5777-A033-4D6F-B604-4A9A1E497330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A128C7F-5997-4E62-A792-920332141BD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -99,7 +99,7 @@
     <t>SỐ ĐNTT-FMS</t>
   </si>
   <si>
-    <t>SỐ TIỀN99</t>
+    <t>SỐ TIỀN</t>
   </si>
 </sst>
 </file>
@@ -525,7 +525,7 @@
     <col min="5" max="5" width="20.5546875" style="2" customWidth="1"/>
     <col min="6" max="6" width="21.88671875" style="2" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="4.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.88671875" style="2" customWidth="1"/>
     <col min="9" max="9" width="17.77734375" style="1" customWidth="1"/>
     <col min="10" max="10" width="20.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22.109375" style="1" customWidth="1"/>

</xml_diff>